<commit_message>
Add CO2 co-benefits, use total rather than annual costs and emissions
</commit_message>
<xml_diff>
--- a/input_data_example.xlsx
+++ b/input_data_example.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\romesh\projects\analyses\carbomica\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BCDB36CA-70F6-4162-9434-B25D4AAF06B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5B40403-0CAE-4BA7-91AF-B3A46FEF8DA9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11670" yWindow="3765" windowWidth="26235" windowHeight="14760" firstSheet="3" activeTab="5" xr2:uid="{0286FA47-14CE-4473-A2C3-5B41DC540DBC}"/>
+    <workbookView xWindow="1950" yWindow="2970" windowWidth="26835" windowHeight="15315" firstSheet="2" activeTab="4" xr2:uid="{0286FA47-14CE-4473-A2C3-5B41DC540DBC}"/>
   </bookViews>
   <sheets>
     <sheet name="Contents" sheetId="10" r:id="rId1"/>
@@ -220,7 +220,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="72">
   <si>
     <t>facilities</t>
   </si>
@@ -556,6 +556,18 @@
   </si>
   <si>
     <t>Improved air quality</t>
+  </si>
+  <si>
+    <t>tree_planting</t>
+  </si>
+  <si>
+    <t>Tree Planting</t>
+  </si>
+  <si>
+    <t>Carbon sequestration, improved air quality, enhanced biodiversity</t>
+  </si>
+  <si>
+    <t>Additional annual CO2 reduction</t>
   </si>
 </sst>
 </file>
@@ -1653,7 +1665,8 @@
     <col min="8" max="8" width="22.28515625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="31.28515625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="29.140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="14" width="6.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="14" width="6.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:304" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -1698,7 +1711,7 @@
       </c>
       <c r="K1" s="2" t="str">
         <f>IF(interventions!$A11&lt;&gt;"",interventions!$A11&amp;"_cost","")</f>
-        <v/>
+        <v>tree_planting_cost</v>
       </c>
       <c r="L1" s="2" t="str">
         <f>IF(interventions!$A12&lt;&gt;"",interventions!$A12&amp;"_cost","")</f>
@@ -2915,21 +2928,11 @@
         <v>800</v>
       </c>
       <c r="K2" s="1">
-        <f>'implementation costs'!K2/10</f>
-        <v>0</v>
-      </c>
-      <c r="L2" s="1">
-        <f>'implementation costs'!L2/10</f>
-        <v>0</v>
-      </c>
-      <c r="M2" s="1">
-        <f>'implementation costs'!M2/10</f>
-        <v>0</v>
-      </c>
-      <c r="N2" s="1">
-        <f>'implementation costs'!N2/10</f>
-        <v>0</v>
-      </c>
+        <v>1500</v>
+      </c>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
     </row>
     <row r="3" spans="1:304" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="str">
@@ -9359,16 +9362,17 @@
   <sheetPr>
     <tabColor theme="5"/>
   </sheetPr>
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="35.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="32" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.28515625" customWidth="1"/>
-    <col min="4" max="4" width="26.28515625" customWidth="1"/>
+    <col min="3" max="3" width="30.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="19.28515625" customWidth="1"/>
+    <col min="5" max="5" width="26.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>1</v>
       </c>
@@ -9376,115 +9380,135 @@
         <v>2</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>42</v>
       </c>
       <c r="B2" t="s">
         <v>51</v>
       </c>
-      <c r="C2" s="14">
+      <c r="D2" s="14">
         <v>100</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>43</v>
       </c>
       <c r="B3" t="s">
         <v>52</v>
       </c>
-      <c r="C3" s="14">
+      <c r="D3" s="14">
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>44</v>
       </c>
       <c r="B4" t="s">
         <v>53</v>
       </c>
-      <c r="C4" s="14">
+      <c r="D4" s="14">
         <v>300</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>45</v>
       </c>
       <c r="B5" t="s">
         <v>54</v>
       </c>
-      <c r="C5" s="14">
+      <c r="D5" s="14">
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>46</v>
       </c>
       <c r="B6" t="s">
         <v>55</v>
       </c>
-      <c r="C6" s="14">
+      <c r="D6" s="14">
         <v>500</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>47</v>
       </c>
       <c r="B7" t="s">
         <v>56</v>
       </c>
-      <c r="C7" s="14">
+      <c r="D7" s="14">
         <v>600</v>
       </c>
-      <c r="D7" t="s">
+      <c r="E7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>48</v>
       </c>
       <c r="B8" t="s">
         <v>57</v>
       </c>
-      <c r="C8" s="14">
+      <c r="D8" s="14">
         <v>700</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>49</v>
       </c>
       <c r="B9" t="s">
         <v>58</v>
       </c>
-      <c r="C9" s="14">
+      <c r="D9" s="14">
         <v>800</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>50</v>
       </c>
       <c r="B10" t="s">
         <v>59</v>
       </c>
-      <c r="C10" s="14">
+      <c r="D10" s="14">
         <v>900</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C11">
+        <v>20000</v>
+      </c>
+      <c r="D11" s="14">
+        <v>-2000</v>
+      </c>
+      <c r="E11" t="s">
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -10861,7 +10885,7 @@
     <row r="11" spans="1:288" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="str">
         <f>IF(interventions!$A11&lt;&gt;"",interventions!$A11,"")</f>
-        <v/>
+        <v>tree_planting</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>
@@ -12919,7 +12943,7 @@
       </c>
       <c r="K1" s="2" t="str">
         <f>IF(interventions!$A11&lt;&gt;"",interventions!$A11&amp;"_effect","")</f>
-        <v/>
+        <v>tree_planting_effect</v>
       </c>
       <c r="L1" s="2" t="str">
         <f>IF(interventions!$A12&lt;&gt;"",interventions!$A12&amp;"_effect","")</f>
@@ -16040,7 +16064,7 @@
       </c>
       <c r="K1" s="2" t="str">
         <f>IF(interventions!$A11&lt;&gt;"",interventions!$A11&amp;"_cost","")</f>
-        <v/>
+        <v>tree_planting_cost</v>
       </c>
       <c r="L1" s="2" t="str">
         <f>IF(interventions!$A12&lt;&gt;"",interventions!$A12&amp;"_cost","")</f>
@@ -17247,7 +17271,9 @@
       <c r="J2" s="1">
         <v>8000</v>
       </c>
-      <c r="K2" s="1"/>
+      <c r="K2" s="1">
+        <v>50000</v>
+      </c>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
       <c r="N2" s="1"/>

</xml_diff>